<commit_message>
power bi folder init
</commit_message>
<xml_diff>
--- a/Excel/2. Dataset/M1_Excel_Training_Dataset.xlsx
+++ b/Excel/2. Dataset/M1_Excel_Training_Dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://p211-my.sharepoint.com/personal/gazala_fathima_talenciaglobal_com/Documents/1.TalenciaGlobal/Excel/SRM-EXCEL/RAW/Module 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanja\Desktop\STEP\Excel\2. Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B0F58F8B-A5AA-4D7F-B1A0-059E3F5D58D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B3E2EB-1803-441B-9547-AACF8632349E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572F0575-2E6A-463C-B8E1-D5F39BEC2A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9560" yWindow="0" windowWidth="9730" windowHeight="11370" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee_Master" sheetId="1" r:id="rId1"/>
@@ -4545,28 +4545,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S154"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="22.21875" customWidth="1"/>
+    <col min="10" max="10" width="22.1796875" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="20.77734375" customWidth="1"/>
-    <col min="18" max="18" width="10.109375" customWidth="1"/>
+    <col min="17" max="17" width="20.81640625" customWidth="1"/>
+    <col min="18" max="18" width="10.08984375" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>19</v>
       </c>
@@ -4684,7 +4684,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>34</v>
       </c>
@@ -4743,7 +4743,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>47</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>59</v>
       </c>
@@ -4861,7 +4861,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>70</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>80</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>87</v>
       </c>
@@ -5034,7 +5034,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>94</v>
       </c>
@@ -5093,7 +5093,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>105</v>
       </c>
@@ -5152,7 +5152,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>110</v>
       </c>
@@ -5211,7 +5211,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>118</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>130</v>
       </c>
@@ -5329,7 +5329,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>140</v>
       </c>
@@ -5388,7 +5388,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>150</v>
       </c>
@@ -5447,7 +5447,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
         <v>157</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>165</v>
       </c>
@@ -5561,7 +5561,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>172</v>
       </c>
@@ -5620,7 +5620,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19" s="11" t="s">
         <v>180</v>
       </c>
@@ -5679,7 +5679,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
         <v>186</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" s="11" t="s">
         <v>192</v>
       </c>
@@ -5797,7 +5797,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22" s="11" t="s">
         <v>200</v>
       </c>
@@ -5856,7 +5856,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
         <v>207</v>
       </c>
@@ -5915,7 +5915,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" s="11" t="s">
         <v>216</v>
       </c>
@@ -5974,7 +5974,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
         <v>222</v>
       </c>
@@ -6033,7 +6033,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26" s="11" t="s">
         <v>229</v>
       </c>
@@ -6088,7 +6088,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
         <v>236</v>
       </c>
@@ -6147,7 +6147,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" s="11" t="s">
         <v>242</v>
       </c>
@@ -6206,7 +6206,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" s="11" t="s">
         <v>248</v>
       </c>
@@ -6265,7 +6265,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30" s="11" t="s">
         <v>255</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31" s="11" t="s">
         <v>259</v>
       </c>
@@ -6383,7 +6383,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A32" s="11" t="s">
         <v>264</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A33" s="11" t="s">
         <v>270</v>
       </c>
@@ -6501,7 +6501,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A34" s="11" t="s">
         <v>274</v>
       </c>
@@ -6560,7 +6560,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
         <v>280</v>
       </c>
@@ -6619,7 +6619,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
         <v>286</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
         <v>290</v>
       </c>
@@ -6733,7 +6733,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A38" s="11" t="s">
         <v>295</v>
       </c>
@@ -6792,7 +6792,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
         <v>301</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
         <v>306</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
         <v>311</v>
       </c>
@@ -6969,7 +6969,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
         <v>315</v>
       </c>
@@ -7028,7 +7028,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
         <v>321</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A44" s="11" t="s">
         <v>326</v>
       </c>
@@ -7146,7 +7146,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
         <v>333</v>
       </c>
@@ -7205,7 +7205,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A46" s="11" t="s">
         <v>338</v>
       </c>
@@ -7264,7 +7264,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>343</v>
       </c>
@@ -7323,7 +7323,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A48" s="11" t="s">
         <v>348</v>
       </c>
@@ -7382,7 +7382,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
         <v>353</v>
       </c>
@@ -7441,7 +7441,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A50" s="11" t="s">
         <v>358</v>
       </c>
@@ -7500,7 +7500,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A51" s="11" t="s">
         <v>363</v>
       </c>
@@ -7559,7 +7559,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A52" s="11" t="s">
         <v>368</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A53" s="11" t="s">
         <v>372</v>
       </c>
@@ -7677,7 +7677,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A54" s="11" t="s">
         <v>377</v>
       </c>
@@ -7736,7 +7736,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A55" s="11" t="s">
         <v>383</v>
       </c>
@@ -7795,7 +7795,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A56" s="11" t="s">
         <v>387</v>
       </c>
@@ -7850,7 +7850,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A57" s="11" t="s">
         <v>393</v>
       </c>
@@ -7909,7 +7909,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A58" s="11" t="s">
         <v>399</v>
       </c>
@@ -7968,7 +7968,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A59" s="11" t="s">
         <v>404</v>
       </c>
@@ -8027,7 +8027,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A60" s="11" t="s">
         <v>409</v>
       </c>
@@ -8086,7 +8086,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A61" s="11" t="s">
         <v>413</v>
       </c>
@@ -8145,7 +8145,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A62" s="11" t="s">
         <v>419</v>
       </c>
@@ -8204,7 +8204,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A63" s="11" t="s">
         <v>424</v>
       </c>
@@ -8263,7 +8263,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A64" s="11" t="s">
         <v>431</v>
       </c>
@@ -8322,7 +8322,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A65" s="11" t="s">
         <v>436</v>
       </c>
@@ -8381,7 +8381,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A66" s="11" t="s">
         <v>442</v>
       </c>
@@ -8436,7 +8436,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A67" s="11" t="s">
         <v>448</v>
       </c>
@@ -8495,7 +8495,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A68" s="11" t="s">
         <v>454</v>
       </c>
@@ -8554,7 +8554,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A69" s="11" t="s">
         <v>459</v>
       </c>
@@ -8613,7 +8613,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A70" s="11" t="s">
         <v>465</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>469</v>
       </c>
@@ -8731,7 +8731,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A72" s="11" t="s">
         <v>473</v>
       </c>
@@ -8790,7 +8790,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
         <v>477</v>
       </c>
@@ -8849,7 +8849,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A74" s="11" t="s">
         <v>481</v>
       </c>
@@ -8908,7 +8908,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A75" s="11" t="s">
         <v>483</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A76" s="11" t="s">
         <v>488</v>
       </c>
@@ -9022,7 +9022,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A77" s="11" t="s">
         <v>495</v>
       </c>
@@ -9081,7 +9081,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A78" s="11" t="s">
         <v>499</v>
       </c>
@@ -9140,7 +9140,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A79" s="11" t="s">
         <v>503</v>
       </c>
@@ -9199,7 +9199,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A80" s="11" t="s">
         <v>509</v>
       </c>
@@ -9258,7 +9258,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A81" s="11" t="s">
         <v>513</v>
       </c>
@@ -9317,7 +9317,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A82" s="11" t="s">
         <v>516</v>
       </c>
@@ -9376,7 +9376,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A83" s="11" t="s">
         <v>520</v>
       </c>
@@ -9435,7 +9435,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A84" s="11" t="s">
         <v>524</v>
       </c>
@@ -9494,7 +9494,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A85" s="11" t="s">
         <v>529</v>
       </c>
@@ -9553,7 +9553,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A86" s="11" t="s">
         <v>531</v>
       </c>
@@ -9608,7 +9608,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A87" s="11" t="s">
         <v>535</v>
       </c>
@@ -9667,7 +9667,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A88" s="11" t="s">
         <v>539</v>
       </c>
@@ -9726,7 +9726,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A89" s="11" t="s">
         <v>543</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A90" s="11" t="s">
         <v>547</v>
       </c>
@@ -9844,7 +9844,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A91" s="11" t="s">
         <v>552</v>
       </c>
@@ -9903,7 +9903,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A92" s="11" t="s">
         <v>556</v>
       </c>
@@ -9962,7 +9962,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A93" s="11" t="s">
         <v>561</v>
       </c>
@@ -10021,7 +10021,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A94" s="11" t="s">
         <v>565</v>
       </c>
@@ -10080,7 +10080,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A95" s="11" t="s">
         <v>569</v>
       </c>
@@ -10139,7 +10139,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A96" s="11" t="s">
         <v>573</v>
       </c>
@@ -10194,7 +10194,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A97" s="11" t="s">
         <v>578</v>
       </c>
@@ -10253,7 +10253,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A98" s="11" t="s">
         <v>582</v>
       </c>
@@ -10312,7 +10312,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A99" s="11" t="s">
         <v>586</v>
       </c>
@@ -10371,7 +10371,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A100" s="11" t="s">
         <v>590</v>
       </c>
@@ -10430,7 +10430,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A101" s="11" t="s">
         <v>594</v>
       </c>
@@ -10489,7 +10489,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A102" s="11" t="s">
         <v>600</v>
       </c>
@@ -10548,7 +10548,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A103" s="11" t="s">
         <v>604</v>
       </c>
@@ -10607,7 +10607,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A104" s="11" t="s">
         <v>609</v>
       </c>
@@ -10666,7 +10666,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A105" s="11" t="s">
         <v>613</v>
       </c>
@@ -10725,7 +10725,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A106" s="11" t="s">
         <v>618</v>
       </c>
@@ -10780,7 +10780,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A107" s="11" t="s">
         <v>623</v>
       </c>
@@ -10839,7 +10839,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A108" s="11" t="s">
         <v>627</v>
       </c>
@@ -10898,7 +10898,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A109" s="11" t="s">
         <v>631</v>
       </c>
@@ -10957,7 +10957,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A110" s="11" t="s">
         <v>635</v>
       </c>
@@ -11016,7 +11016,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A111" s="11" t="s">
         <v>639</v>
       </c>
@@ -11075,7 +11075,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A112" s="11" t="s">
         <v>644</v>
       </c>
@@ -11134,7 +11134,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A113" s="11" t="s">
         <v>648</v>
       </c>
@@ -11193,7 +11193,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A114" s="11" t="s">
         <v>652</v>
       </c>
@@ -11252,7 +11252,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A115" s="11" t="s">
         <v>656</v>
       </c>
@@ -11311,7 +11311,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A116" s="11" t="s">
         <v>660</v>
       </c>
@@ -11366,7 +11366,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A117" s="11" t="s">
         <v>664</v>
       </c>
@@ -11425,7 +11425,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A118" s="11" t="s">
         <v>668</v>
       </c>
@@ -11484,7 +11484,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A119" s="11" t="s">
         <v>673</v>
       </c>
@@ -11543,7 +11543,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A120" s="11" t="s">
         <v>677</v>
       </c>
@@ -11602,7 +11602,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A121" s="11" t="s">
         <v>681</v>
       </c>
@@ -11661,7 +11661,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A122" s="11" t="s">
         <v>686</v>
       </c>
@@ -11720,7 +11720,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A123" s="11" t="s">
         <v>690</v>
       </c>
@@ -11779,7 +11779,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A124" s="11" t="s">
         <v>694</v>
       </c>
@@ -11838,7 +11838,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A125" s="11" t="s">
         <v>698</v>
       </c>
@@ -11897,7 +11897,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A126" s="11" t="s">
         <v>700</v>
       </c>
@@ -11952,7 +11952,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A127" s="11" t="s">
         <v>705</v>
       </c>
@@ -12011,7 +12011,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A128" s="11" t="s">
         <v>710</v>
       </c>
@@ -12070,7 +12070,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A129" s="11" t="s">
         <v>714</v>
       </c>
@@ -12129,7 +12129,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A130" s="11" t="s">
         <v>719</v>
       </c>
@@ -12188,7 +12188,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A131" s="11" t="s">
         <v>723</v>
       </c>
@@ -12247,7 +12247,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A132" s="11" t="s">
         <v>727</v>
       </c>
@@ -12306,7 +12306,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A133" s="11" t="s">
         <v>732</v>
       </c>
@@ -12365,7 +12365,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A134" s="11" t="s">
         <v>736</v>
       </c>
@@ -12424,7 +12424,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A135" s="11" t="s">
         <v>740</v>
       </c>
@@ -12483,7 +12483,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A136" s="11" t="s">
         <v>744</v>
       </c>
@@ -12538,7 +12538,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A137" s="11" t="s">
         <v>749</v>
       </c>
@@ -12597,7 +12597,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A138" s="11" t="s">
         <v>753</v>
       </c>
@@ -12656,7 +12656,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A139" s="11" t="s">
         <v>758</v>
       </c>
@@ -12715,7 +12715,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A140" s="11" t="s">
         <v>762</v>
       </c>
@@ -12774,7 +12774,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A141" s="11" t="s">
         <v>766</v>
       </c>
@@ -12833,7 +12833,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A142" s="11" t="s">
         <v>770</v>
       </c>
@@ -12892,7 +12892,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A143" s="11" t="s">
         <v>774</v>
       </c>
@@ -12951,7 +12951,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A144" s="11" t="s">
         <v>778</v>
       </c>
@@ -13010,7 +13010,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A145" s="11" t="s">
         <v>782</v>
       </c>
@@ -13069,7 +13069,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A146" s="11" t="s">
         <v>786</v>
       </c>
@@ -13124,7 +13124,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A147" s="11" t="s">
         <v>791</v>
       </c>
@@ -13183,7 +13183,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A148" s="11" t="s">
         <v>795</v>
       </c>
@@ -13242,7 +13242,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A149" s="11" t="s">
         <v>799</v>
       </c>
@@ -13301,7 +13301,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A150" s="11" t="s">
         <v>803</v>
       </c>
@@ -13360,7 +13360,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A151" s="11" t="s">
         <v>807</v>
       </c>
@@ -13419,7 +13419,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A152" s="11" t="s">
         <v>70</v>
       </c>
@@ -13474,7 +13474,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A153" s="11" t="s">
         <v>259</v>
       </c>
@@ -13533,7 +13533,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A154" s="16" t="s">
         <v>70</v>
       </c>
@@ -13600,12 +13600,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>811</v>
       </c>
@@ -13622,7 +13622,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>816</v>
       </c>
@@ -13639,7 +13639,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>817</v>
       </c>
@@ -13656,7 +13656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>818</v>
       </c>
@@ -13673,7 +13673,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>819</v>
       </c>
@@ -13690,7 +13690,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>820</v>
       </c>
@@ -13707,7 +13707,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>821</v>
       </c>
@@ -13733,12 +13733,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
@@ -13758,7 +13758,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -13779,7 +13779,7 @@
         <v>23500000</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>99</v>
       </c>
@@ -13800,7 +13800,7 @@
         <v>9500000</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
@@ -13821,7 +13821,7 @@
         <v>39000000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>75</v>
       </c>
@@ -13842,7 +13842,7 @@
         <v>15000000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>330</v>
       </c>
@@ -13863,7 +13863,7 @@
         <v>19000000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>83</v>
       </c>
@@ -13893,12 +13893,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H201"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>827</v>
       </c>
@@ -13924,7 +13924,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>832</v>
       </c>
@@ -13950,7 +13950,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>835</v>
       </c>
@@ -13976,7 +13976,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>838</v>
       </c>
@@ -14002,7 +14002,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>840</v>
       </c>
@@ -14028,7 +14028,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>843</v>
       </c>
@@ -14054,7 +14054,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>845</v>
       </c>
@@ -14080,7 +14080,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>846</v>
       </c>
@@ -14106,7 +14106,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>848</v>
       </c>
@@ -14132,7 +14132,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>849</v>
       </c>
@@ -14158,7 +14158,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>851</v>
       </c>
@@ -14184,7 +14184,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>852</v>
       </c>
@@ -14210,7 +14210,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>854</v>
       </c>
@@ -14236,7 +14236,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>856</v>
       </c>
@@ -14262,7 +14262,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>857</v>
       </c>
@@ -14288,7 +14288,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>859</v>
       </c>
@@ -14314,7 +14314,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>860</v>
       </c>
@@ -14340,7 +14340,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>861</v>
       </c>
@@ -14366,7 +14366,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>863</v>
       </c>
@@ -14392,7 +14392,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>864</v>
       </c>
@@ -14418,7 +14418,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>865</v>
       </c>
@@ -14444,7 +14444,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>866</v>
       </c>
@@ -14470,7 +14470,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>867</v>
       </c>
@@ -14496,7 +14496,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>869</v>
       </c>
@@ -14522,7 +14522,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>870</v>
       </c>
@@ -14548,7 +14548,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>872</v>
       </c>
@@ -14574,7 +14574,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>873</v>
       </c>
@@ -14600,7 +14600,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>874</v>
       </c>
@@ -14626,7 +14626,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>875</v>
       </c>
@@ -14652,7 +14652,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>876</v>
       </c>
@@ -14678,7 +14678,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>877</v>
       </c>
@@ -14704,7 +14704,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>878</v>
       </c>
@@ -14730,7 +14730,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>879</v>
       </c>
@@ -14756,7 +14756,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>880</v>
       </c>
@@ -14782,7 +14782,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>881</v>
       </c>
@@ -14808,7 +14808,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>882</v>
       </c>
@@ -14834,7 +14834,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>883</v>
       </c>
@@ -14860,7 +14860,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>884</v>
       </c>
@@ -14886,7 +14886,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>886</v>
       </c>
@@ -14912,7 +14912,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>887</v>
       </c>
@@ -14938,7 +14938,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>888</v>
       </c>
@@ -14964,7 +14964,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>890</v>
       </c>
@@ -14990,7 +14990,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>891</v>
       </c>
@@ -15016,7 +15016,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>892</v>
       </c>
@@ -15042,7 +15042,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>893</v>
       </c>
@@ -15068,7 +15068,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>894</v>
       </c>
@@ -15094,7 +15094,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>895</v>
       </c>
@@ -15120,7 +15120,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>896</v>
       </c>
@@ -15146,7 +15146,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>897</v>
       </c>
@@ -15172,7 +15172,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>898</v>
       </c>
@@ -15198,7 +15198,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>899</v>
       </c>
@@ -15224,7 +15224,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>900</v>
       </c>
@@ -15250,7 +15250,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>901</v>
       </c>
@@ -15276,7 +15276,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>902</v>
       </c>
@@ -15302,7 +15302,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>903</v>
       </c>
@@ -15328,7 +15328,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>904</v>
       </c>
@@ -15354,7 +15354,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>905</v>
       </c>
@@ -15380,7 +15380,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>906</v>
       </c>
@@ -15406,7 +15406,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>907</v>
       </c>
@@ -15432,7 +15432,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>908</v>
       </c>
@@ -15458,7 +15458,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>909</v>
       </c>
@@ -15484,7 +15484,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>910</v>
       </c>
@@ -15510,7 +15510,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>911</v>
       </c>
@@ -15536,7 +15536,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>912</v>
       </c>
@@ -15562,7 +15562,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>913</v>
       </c>
@@ -15588,7 +15588,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>914</v>
       </c>
@@ -15614,7 +15614,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>915</v>
       </c>
@@ -15640,7 +15640,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>916</v>
       </c>
@@ -15666,7 +15666,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>917</v>
       </c>
@@ -15692,7 +15692,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>918</v>
       </c>
@@ -15718,7 +15718,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>919</v>
       </c>
@@ -15744,7 +15744,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>920</v>
       </c>
@@ -15770,7 +15770,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>921</v>
       </c>
@@ -15796,7 +15796,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>922</v>
       </c>
@@ -15822,7 +15822,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>923</v>
       </c>
@@ -15848,7 +15848,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>924</v>
       </c>
@@ -15874,7 +15874,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>925</v>
       </c>
@@ -15900,7 +15900,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>926</v>
       </c>
@@ -15926,7 +15926,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>927</v>
       </c>
@@ -15952,7 +15952,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>928</v>
       </c>
@@ -15978,7 +15978,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>929</v>
       </c>
@@ -16004,7 +16004,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>930</v>
       </c>
@@ -16030,7 +16030,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>931</v>
       </c>
@@ -16056,7 +16056,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>932</v>
       </c>
@@ -16082,7 +16082,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>933</v>
       </c>
@@ -16108,7 +16108,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>934</v>
       </c>
@@ -16134,7 +16134,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>935</v>
       </c>
@@ -16160,7 +16160,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>936</v>
       </c>
@@ -16186,7 +16186,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>937</v>
       </c>
@@ -16212,7 +16212,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>938</v>
       </c>
@@ -16238,7 +16238,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>939</v>
       </c>
@@ -16264,7 +16264,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>940</v>
       </c>
@@ -16290,7 +16290,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>941</v>
       </c>
@@ -16316,7 +16316,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>942</v>
       </c>
@@ -16342,7 +16342,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>943</v>
       </c>
@@ -16368,7 +16368,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>944</v>
       </c>
@@ -16394,7 +16394,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>945</v>
       </c>
@@ -16420,7 +16420,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>946</v>
       </c>
@@ -16446,7 +16446,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>947</v>
       </c>
@@ -16472,7 +16472,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>948</v>
       </c>
@@ -16498,7 +16498,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>949</v>
       </c>
@@ -16524,7 +16524,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>950</v>
       </c>
@@ -16550,7 +16550,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>951</v>
       </c>
@@ -16576,7 +16576,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>952</v>
       </c>
@@ -16602,7 +16602,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>953</v>
       </c>
@@ -16628,7 +16628,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>954</v>
       </c>
@@ -16654,7 +16654,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>955</v>
       </c>
@@ -16680,7 +16680,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>956</v>
       </c>
@@ -16706,7 +16706,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>957</v>
       </c>
@@ -16732,7 +16732,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>958</v>
       </c>
@@ -16758,7 +16758,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>959</v>
       </c>
@@ -16784,7 +16784,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>960</v>
       </c>
@@ -16810,7 +16810,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>961</v>
       </c>
@@ -16836,7 +16836,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>962</v>
       </c>
@@ -16862,7 +16862,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>963</v>
       </c>
@@ -16888,7 +16888,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>964</v>
       </c>
@@ -16914,7 +16914,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>965</v>
       </c>
@@ -16940,7 +16940,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>966</v>
       </c>
@@ -16966,7 +16966,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>967</v>
       </c>
@@ -16992,7 +16992,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>968</v>
       </c>
@@ -17018,7 +17018,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>969</v>
       </c>
@@ -17044,7 +17044,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>970</v>
       </c>
@@ -17070,7 +17070,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>971</v>
       </c>
@@ -17096,7 +17096,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>972</v>
       </c>
@@ -17122,7 +17122,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>973</v>
       </c>
@@ -17148,7 +17148,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>974</v>
       </c>
@@ -17174,7 +17174,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>975</v>
       </c>
@@ -17200,7 +17200,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>976</v>
       </c>
@@ -17226,7 +17226,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>977</v>
       </c>
@@ -17252,7 +17252,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>978</v>
       </c>
@@ -17278,7 +17278,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>979</v>
       </c>
@@ -17304,7 +17304,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>980</v>
       </c>
@@ -17330,7 +17330,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>981</v>
       </c>
@@ -17356,7 +17356,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>982</v>
       </c>
@@ -17382,7 +17382,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>983</v>
       </c>
@@ -17408,7 +17408,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>984</v>
       </c>
@@ -17434,7 +17434,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>985</v>
       </c>
@@ -17460,7 +17460,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>986</v>
       </c>
@@ -17486,7 +17486,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>987</v>
       </c>
@@ -17512,7 +17512,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>988</v>
       </c>
@@ -17538,7 +17538,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>989</v>
       </c>
@@ -17564,7 +17564,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>990</v>
       </c>
@@ -17590,7 +17590,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>991</v>
       </c>
@@ -17616,7 +17616,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>992</v>
       </c>
@@ -17642,7 +17642,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>993</v>
       </c>
@@ -17668,7 +17668,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>994</v>
       </c>
@@ -17694,7 +17694,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>995</v>
       </c>
@@ -17720,7 +17720,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>996</v>
       </c>
@@ -17746,7 +17746,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>997</v>
       </c>
@@ -17772,7 +17772,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>998</v>
       </c>
@@ -17798,7 +17798,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>999</v>
       </c>
@@ -17824,7 +17824,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>1000</v>
       </c>
@@ -17850,7 +17850,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>1001</v>
       </c>
@@ -17876,7 +17876,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>1002</v>
       </c>
@@ -17902,7 +17902,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>1003</v>
       </c>
@@ -17928,7 +17928,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>1004</v>
       </c>
@@ -17954,7 +17954,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>1005</v>
       </c>
@@ -17980,7 +17980,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>1006</v>
       </c>
@@ -18006,7 +18006,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>1007</v>
       </c>
@@ -18032,7 +18032,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>1008</v>
       </c>
@@ -18058,7 +18058,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>1009</v>
       </c>
@@ -18084,7 +18084,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>1010</v>
       </c>
@@ -18110,7 +18110,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>1011</v>
       </c>
@@ -18136,7 +18136,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>1012</v>
       </c>
@@ -18162,7 +18162,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>1013</v>
       </c>
@@ -18188,7 +18188,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>1014</v>
       </c>
@@ -18214,7 +18214,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>1015</v>
       </c>
@@ -18240,7 +18240,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>1016</v>
       </c>
@@ -18266,7 +18266,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>1017</v>
       </c>
@@ -18292,7 +18292,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>1018</v>
       </c>
@@ -18318,7 +18318,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>1019</v>
       </c>
@@ -18344,7 +18344,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>1020</v>
       </c>
@@ -18370,7 +18370,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>1021</v>
       </c>
@@ -18396,7 +18396,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>1022</v>
       </c>
@@ -18422,7 +18422,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>1023</v>
       </c>
@@ -18448,7 +18448,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>1024</v>
       </c>
@@ -18474,7 +18474,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>1025</v>
       </c>
@@ -18500,7 +18500,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>1026</v>
       </c>
@@ -18526,7 +18526,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>1027</v>
       </c>
@@ -18552,7 +18552,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>1028</v>
       </c>
@@ -18578,7 +18578,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>1029</v>
       </c>
@@ -18604,7 +18604,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>1030</v>
       </c>
@@ -18630,7 +18630,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>1031</v>
       </c>
@@ -18656,7 +18656,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>1032</v>
       </c>
@@ -18682,7 +18682,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>1033</v>
       </c>
@@ -18708,7 +18708,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>1034</v>
       </c>
@@ -18734,7 +18734,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>1035</v>
       </c>
@@ -18760,7 +18760,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>1036</v>
       </c>
@@ -18786,7 +18786,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>1037</v>
       </c>
@@ -18812,7 +18812,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>1038</v>
       </c>
@@ -18838,7 +18838,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>1039</v>
       </c>
@@ -18864,7 +18864,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>1040</v>
       </c>
@@ -18890,7 +18890,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>1041</v>
       </c>
@@ -18916,7 +18916,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>1042</v>
       </c>
@@ -18942,7 +18942,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>1043</v>
       </c>
@@ -18968,7 +18968,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>1044</v>
       </c>
@@ -18994,7 +18994,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>1045</v>
       </c>
@@ -19020,7 +19020,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>1046</v>
       </c>
@@ -19046,7 +19046,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>1047</v>
       </c>
@@ -19072,7 +19072,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>1048</v>
       </c>
@@ -19098,7 +19098,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>1049</v>
       </c>
@@ -19134,12 +19134,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F45"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1050</v>
       </c>
@@ -19159,7 +19159,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19179,7 +19179,7 @@
         <v>6058759</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19199,7 +19199,7 @@
         <v>4693149</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19219,7 +19219,7 @@
         <v>3916518</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19239,7 +19239,7 @@
         <v>6163305</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19259,7 +19259,7 @@
         <v>1065684</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19279,7 +19279,7 @@
         <v>11238365</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19299,7 +19299,7 @@
         <v>550367</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1055</v>
       </c>
@@ -19319,7 +19319,7 @@
         <v>3075370</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19339,7 +19339,7 @@
         <v>3715791</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19359,7 +19359,7 @@
         <v>1273600</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19379,7 +19379,7 @@
         <v>4739936</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19399,7 +19399,7 @@
         <v>39945997</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19419,7 +19419,7 @@
         <v>2031345</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19439,7 +19439,7 @@
         <v>571701</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19459,7 +19459,7 @@
         <v>1622562</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>1064</v>
       </c>
@@ -19479,7 +19479,7 @@
         <v>9853408</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19499,7 +19499,7 @@
         <v>11252086</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19519,7 +19519,7 @@
         <v>12325876</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19539,7 +19539,7 @@
         <v>699641</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19559,7 +19559,7 @@
         <v>5376504</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19579,7 +19579,7 @@
         <v>24734399</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19599,7 +19599,7 @@
         <v>3831679</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19619,7 +19619,7 @@
         <v>8719217</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>1065</v>
       </c>
@@ -19639,7 +19639,7 @@
         <v>2899969</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19659,7 +19659,7 @@
         <v>14818670</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19679,7 +19679,7 @@
         <v>4956115</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19699,7 +19699,7 @@
         <v>2215385</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19719,7 +19719,7 @@
         <v>1233757</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19739,7 +19739,7 @@
         <v>34679195</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19759,7 +19759,7 @@
         <v>2272100</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19779,7 +19779,7 @@
         <v>987369</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>1066</v>
       </c>
@@ -19799,7 +19799,7 @@
         <v>1258942</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19819,7 +19819,7 @@
         <v>571572</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19839,7 +19839,7 @@
         <v>31801760</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19859,7 +19859,7 @@
         <v>4498537</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19879,7 +19879,7 @@
         <v>2101780</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19899,7 +19899,7 @@
         <v>1860063</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19919,7 +19919,7 @@
         <v>375319</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>1067</v>
       </c>
@@ -19939,7 +19939,7 @@
         <v>888862</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>1067</v>
       </c>

</xml_diff>